<commit_message>
Add supermarket sales analysis project
</commit_message>
<xml_diff>
--- a/Supermarket-sales-analysis.xlsx.xlsx
+++ b/Supermarket-sales-analysis.xlsx.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="3" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" firstSheet="3" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Original Sales Data" sheetId="1" r:id="rId1"/>
@@ -240,7 +240,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$₦]#,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -301,6 +301,13 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -528,13 +535,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" pivotButton="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" pivotButton="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="10">
     <dxf>
       <font>
         <b/>
@@ -551,20 +558,19 @@
       </font>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -590,13 +596,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Original Sales Data-style" pivot="0" count="4">
-      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
-      <tableStyleElement type="headerRow" dxfId="6"/>
-      <tableStyleElement type="firstRowStripe" dxfId="5"/>
-      <tableStyleElement type="secondRowStripe" dxfId="4"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="9"/>
+      <tableStyleElement type="headerRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="secondRowStripe" dxfId="6"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -638,7 +660,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -689,7 +710,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -777,7 +797,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -850,7 +869,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -923,7 +941,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -996,7 +1013,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1069,7 +1085,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1142,7 +1157,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1215,7 +1229,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1288,7 +1301,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1361,7 +1373,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1434,7 +1445,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1507,7 +1517,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1580,7 +1589,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1653,7 +1661,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1726,7 +1733,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1799,7 +1805,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1872,7 +1877,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1945,7 +1949,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2018,7 +2021,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2091,7 +2093,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2164,7 +2165,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2237,7 +2237,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2310,7 +2309,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2383,7 +2381,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2456,7 +2453,6 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2546,7 +2542,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2642,7 +2637,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -2721,7 +2715,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="HP" refreshedDate="46319.597532638887" refreshedVersion="6" recordCount="15">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshOnLoad="1" refreshedBy="HP" refreshedDate="46319.643478472222" refreshedVersion="6" recordCount="15">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:I16" sheet="Original Sales Data"/>
   </cacheSource>
@@ -3117,13 +3111,13 @@
     <dataField name="Total Revenue" fld="8" baseField="2" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="2">
+    <format dxfId="5">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -4009,10 +4003,10 @@
   <dimension ref="A1:A1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="66.90625" customWidth="1"/>
+    <col min="1" max="1" width="70.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4020,7 +4014,7 @@
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -4028,7 +4022,7 @@
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
     </row>
-    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -4036,7 +4030,7 @@
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="13" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -4044,7 +4038,7 @@
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
@@ -4052,7 +4046,7 @@
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -4060,7 +4054,7 @@
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" ht="88" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>8</v>
       </c>
@@ -34604,7 +34598,7 @@
     <col min="2" max="2" width="19.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
         <v>20</v>
       </c>

</xml_diff>